<commit_message>
Atualiza Parciais Rodada 15
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_4.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_4.xlsx
@@ -59,10 +59,10 @@
     <t>Jogo 2 (JG2)</t>
   </si>
   <si>
+    <t>TEAM LOPES 99</t>
+  </si>
+  <si>
     <t>LISI GREMISTA</t>
-  </si>
-  <si>
-    <t>TEAM LOPES 99</t>
   </si>
 </sst>
 </file>
@@ -463,10 +463,10 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -475,13 +475,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>61.17</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>48.27</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>12.9</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -504,16 +504,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>48.27</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>61.17</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>-12.9</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -569,10 +569,10 @@
         <v>14</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -581,13 +581,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>58.27</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>39.22</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>19.05</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -610,16 +610,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>39.22</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>58.27</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>-19.05</v>
       </c>
       <c r="J3">
         <v>2</v>

</xml_diff>

<commit_message>
Resultado Final Rodada 15
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_4.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_4.xlsx
@@ -475,13 +475,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>61.17</v>
+        <v>61.169921875</v>
       </c>
       <c r="H2">
-        <v>48.27</v>
+        <v>48.27001953125</v>
       </c>
       <c r="I2">
-        <v>12.9</v>
+        <v>12.89990234375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -507,13 +507,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>48.27</v>
+        <v>48.27001953125</v>
       </c>
       <c r="H3">
-        <v>61.17</v>
+        <v>61.169921875</v>
       </c>
       <c r="I3">
-        <v>-12.9</v>
+        <v>-12.89990234375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -581,13 +581,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>58.27</v>
+        <v>58.27001953125</v>
       </c>
       <c r="H2">
-        <v>39.22</v>
+        <v>39.219970703125</v>
       </c>
       <c r="I2">
-        <v>19.05</v>
+        <v>19.050048828125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -613,13 +613,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>39.22</v>
+        <v>39.219970703125</v>
       </c>
       <c r="H3">
-        <v>58.27</v>
+        <v>58.27001953125</v>
       </c>
       <c r="I3">
-        <v>-19.05</v>
+        <v>-19.050048828125</v>
       </c>
       <c r="J3">
         <v>2</v>

</xml_diff>

<commit_message>
Atualiza Parciais Rodada 16
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_4.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_4.xlsx
@@ -59,10 +59,10 @@
     <t>Jogo 2 (JG2)</t>
   </si>
   <si>
+    <t>LISI GREMISTA</t>
+  </si>
+  <si>
     <t>TEAM LOPES 99</t>
-  </si>
-  <si>
-    <t>LISI GREMISTA</t>
   </si>
 </sst>
 </file>
@@ -472,16 +472,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>61.169921875</v>
+        <v>142.449921875</v>
       </c>
       <c r="H2">
-        <v>48.27001953125</v>
+        <v>136.15001953125</v>
       </c>
       <c r="I2">
-        <v>12.89990234375</v>
+        <v>6.299902343750006</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -495,10 +495,10 @@
         <v>12</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -507,13 +507,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>48.27001953125</v>
+        <v>136.15001953125</v>
       </c>
       <c r="H3">
-        <v>61.169921875</v>
+        <v>142.449921875</v>
       </c>
       <c r="I3">
-        <v>-12.89990234375</v>
+        <v>-6.299902343750006</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -578,16 +578,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>58.27001953125</v>
+        <v>153.509970703125</v>
       </c>
       <c r="H2">
-        <v>39.219970703125</v>
+        <v>141.77001953125</v>
       </c>
       <c r="I2">
-        <v>19.050048828125</v>
+        <v>11.73995117187502</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -601,10 +601,10 @@
         <v>15</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -613,13 +613,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>39.219970703125</v>
+        <v>141.77001953125</v>
       </c>
       <c r="H3">
-        <v>58.27001953125</v>
+        <v>153.509970703125</v>
       </c>
       <c r="I3">
-        <v>-19.050048828125</v>
+        <v>-11.73995117187502</v>
       </c>
       <c r="J3">
         <v>2</v>

</xml_diff>

<commit_message>
Resultado Final Rodada 16
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_4.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_4.xlsx
@@ -475,13 +475,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>142.449921875</v>
+        <v>142.44970703125</v>
       </c>
       <c r="H2">
-        <v>136.15001953125</v>
+        <v>136.14990234375</v>
       </c>
       <c r="I2">
-        <v>6.299902343750006</v>
+        <v>6.2998046875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -507,13 +507,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>136.15001953125</v>
+        <v>136.14990234375</v>
       </c>
       <c r="H3">
-        <v>142.449921875</v>
+        <v>142.44970703125</v>
       </c>
       <c r="I3">
-        <v>-6.299902343750006</v>
+        <v>-6.2998046875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -581,13 +581,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>153.509970703125</v>
+        <v>153.510009765625</v>
       </c>
       <c r="H2">
         <v>141.77001953125</v>
       </c>
       <c r="I2">
-        <v>11.73995117187502</v>
+        <v>11.739990234375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -616,10 +616,10 @@
         <v>141.77001953125</v>
       </c>
       <c r="H3">
-        <v>153.509970703125</v>
+        <v>153.510009765625</v>
       </c>
       <c r="I3">
-        <v>-11.73995117187502</v>
+        <v>-11.739990234375</v>
       </c>
       <c r="J3">
         <v>2</v>

</xml_diff>